<commit_message>
chore(presupuesto): sync disc head printed parts, spring and rod lengths
</commit_message>
<xml_diff>
--- a/presupuesto/MathBot_Presupuesto_SCARA.xlsx
+++ b/presupuesto/MathBot_Presupuesto_SCARA.xlsx
@@ -38,7 +38,7 @@
     <definedName name="RendimientoGH">Supuestos!$C$17</definedName>
     <definedName name="TasaVentasEEUU">Supuestos!$C$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -3843,8 +3843,10 @@
       <c r="Z5" s="27" t="s">
         <v>94</v>
       </c>
-      <c r="AA5" s="28" t="s">
-        <v>95</v>
+      <c r="AA5" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTM usa 400 mm. Con el cabezal de disco v3 bastan 250 mm (NEMA estándar en J2) o 240 mm (NEMA corto): comprar 300 y cortar.</t>
+        </is>
       </c>
       <c r="AB5" s="26">
         <f t="shared" ref="AB5:AB49" si="6">IF(AND(S5="Amazon",ISNUMBER(M5),W5&gt;0),ROUNDUP(G5/N5,0)*M5,0)</f>
@@ -4033,8 +4035,10 @@
       <c r="Z7" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="AA7" s="28" t="s">
-        <v>108</v>
+      <c r="AA7" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTM lo corta a 380 mm para varillas de 400; con varillas de 250 mm cortar a ≈230 mm. El paquete trae 2.</t>
+        </is>
       </c>
       <c r="AB7" s="26">
         <f t="shared" si="6"/>
@@ -5073,8 +5077,10 @@
       <c r="Z18" s="27" t="s">
         <v>172</v>
       </c>
-      <c r="AA18" s="28" t="s">
-        <v>173</v>
+      <c r="AA18" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prestados. Si usan el NEMA corto también en J2 (varillas de 240 mm), bajar a 2 y subir ELE-02 a 2. Confirmar que trae cable.</t>
+        </is>
       </c>
       <c r="AB18" s="26">
         <f t="shared" si="6"/>
@@ -6281,8 +6287,10 @@
       <c r="C32" s="22" t="s">
         <v>255</v>
       </c>
-      <c r="D32" s="22" t="s">
-        <v>256</v>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ø15–16 × 30 mm, alambre 0.5–0.6 (Ø int. ≥ 13.5, sólido ≤ 6 mm)</t>
+        </is>
       </c>
       <c r="E32" s="22" t="s">
         <v>257</v>
@@ -6355,8 +6363,10 @@
       <c r="Z32" s="27" t="s">
         <v>259</v>
       </c>
-      <c r="AA32" s="28" t="s">
-        <v>260</v>
+      <c r="AA32" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Va alrededor del plumón (Ø12): el de Ø10–12 × 20 no entra ni da 18 mm de levante. Ver Cabezal disco/README.md.</t>
+        </is>
       </c>
       <c r="AB32" s="26">
         <f t="shared" si="6"/>
@@ -6374,14 +6384,20 @@
       <c r="B33" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="22" t="s">
-        <v>262</v>
-      </c>
-      <c r="D33" s="22" t="s">
-        <v>263</v>
-      </c>
-      <c r="E33" s="22" t="s">
-        <v>264</v>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tornillería del cabezal A v3</t>
+        </is>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 × M4×35 + tuerca + arandela + fijador de rosca; M3: 4×10, 1×12, 3×20, 1×35, 3×16 avellanados + 11 tuercas</t>
+        </is>
+      </c>
+      <c r="E33" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Placa + separador al J3 Coupler y montaje de las herramientas</t>
+        </is>
       </c>
       <c r="F33" s="21" t="s">
         <v>192</v>
@@ -6443,8 +6459,10 @@
       </c>
       <c r="Y33" s="23"/>
       <c r="Z33" s="21"/>
-      <c r="AA33" s="28" t="s">
-        <v>266</v>
+      <c r="AA33" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El separador del electroimán ahora es impreso (hoja Impresión 3D). Lista por pieza en BRAZO SCARA/DISEÑO FINAL/Cabezal disco/README.md.</t>
+        </is>
       </c>
       <c r="AB33" s="26">
         <f t="shared" si="6"/>
@@ -16233,8 +16251,10 @@
       <c r="A37" s="37">
         <v>25</v>
       </c>
-      <c r="B37" s="37" t="s">
-        <v>413</v>
+      <c r="B37" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Placa trébol del cabezal A v3 (6 mm, PETG)</t>
+        </is>
       </c>
       <c r="C37" s="37" t="s">
         <v>28</v>
@@ -16242,21 +16262,23 @@
       <c r="D37" s="37">
         <v>1</v>
       </c>
-      <c r="E37" s="50"/>
+      <c r="E37" s="50">
+        <v>35.8</v>
+      </c>
       <c r="F37" s="53">
-        <v>30</v>
+        <v>31.5</v>
       </c>
       <c r="G37" s="50">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>31.5</v>
       </c>
       <c r="H37" s="50">
         <f t="shared" si="1"/>
-        <v>2.5641025641025643</v>
+        <v>2.6923076923076925</v>
       </c>
       <c r="I37" s="50">
         <f t="shared" si="2"/>
-        <v>2.5641025641025643</v>
+        <v>2.6923076923076925</v>
       </c>
       <c r="J37" s="36" t="s">
         <v>382</v>
@@ -16266,16 +16288,20 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M37" s="52" t="s">
-        <v>414</v>
+      <c r="M37" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STL en BRAZO SCARA/DISEÑO FINAL/Cabezal disco/STL/02_placa_trebol.stl · boca abajo, sin soportes</t>
+        </is>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" s="37">
         <v>26</v>
       </c>
-      <c r="B38" s="37" t="s">
-        <v>415</v>
+      <c r="B38" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Separador de brida 14 mm (PETG)</t>
+        </is>
       </c>
       <c r="C38" s="37" t="s">
         <v>28</v>
@@ -16283,21 +16309,23 @@
       <c r="D38" s="37">
         <v>1</v>
       </c>
-      <c r="E38" s="50"/>
+      <c r="E38" s="50">
+        <v>9.7</v>
+      </c>
       <c r="F38" s="53">
-        <v>8</v>
+        <v>12.4</v>
       </c>
       <c r="G38" s="50">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>12.4</v>
       </c>
       <c r="H38" s="50">
         <f t="shared" si="1"/>
-        <v>0.68376068376068377</v>
+        <v>1.0598290598290598</v>
       </c>
       <c r="I38" s="50">
         <f t="shared" si="2"/>
-        <v>0.68376068376068377</v>
+        <v>1.0598290598290598</v>
       </c>
       <c r="J38" s="36" t="s">
         <v>382</v>
@@ -16307,16 +16335,20 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M38" s="52" t="s">
-        <v>414</v>
+      <c r="M38" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STL en BRAZO SCARA/DISEÑO FINAL/Cabezal disco/STL/01_separador_brida.stl · baja la placa 14 mm para no chocar con la cubierta del brazo 2</t>
+        </is>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" s="37">
         <v>27</v>
       </c>
-      <c r="B39" s="37" t="s">
-        <v>416</v>
+      <c r="B39" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Soporte plumón/servo + puente + collar (PETG, 3 piezas)</t>
+        </is>
       </c>
       <c r="C39" s="37" t="s">
         <v>28</v>
@@ -16324,21 +16356,23 @@
       <c r="D39" s="37">
         <v>1</v>
       </c>
-      <c r="E39" s="50"/>
+      <c r="E39" s="50">
+        <v>9.7</v>
+      </c>
       <c r="F39" s="53">
-        <v>5</v>
+        <v>11.8</v>
       </c>
       <c r="G39" s="50">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>11.8</v>
       </c>
       <c r="H39" s="50">
         <f t="shared" si="1"/>
-        <v>0.42735042735042739</v>
+        <v>1.0085470085470087</v>
       </c>
       <c r="I39" s="50">
         <f t="shared" si="2"/>
-        <v>0.42735042735042739</v>
+        <v>1.0085470085470087</v>
       </c>
       <c r="J39" s="36" t="s">
         <v>382</v>
@@ -16348,16 +16382,20 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M39" s="52" t="s">
-        <v>414</v>
+      <c r="M39" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STL en BRAZO SCARA/DISEÑO FINAL/Cabezal disco/STL/03, 04 y 05 · gramos de las tres piezas</t>
+        </is>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="37">
         <v>28</v>
       </c>
-      <c r="B40" s="37" t="s">
-        <v>417</v>
+      <c r="B40" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Separador del electroimán con copa (PLA+)</t>
+        </is>
       </c>
       <c r="C40" s="37" t="s">
         <v>28</v>
@@ -16365,21 +16403,23 @@
       <c r="D40" s="37">
         <v>1</v>
       </c>
-      <c r="E40" s="50"/>
+      <c r="E40" s="50">
+        <v>6.5</v>
+      </c>
       <c r="F40" s="53">
-        <v>3</v>
+        <v>6.0</v>
       </c>
       <c r="G40" s="50">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>6.0</v>
       </c>
       <c r="H40" s="50">
         <f t="shared" si="1"/>
-        <v>0.25641025641025644</v>
+        <v>0.5128205128205129</v>
       </c>
       <c r="I40" s="50">
         <f t="shared" si="2"/>
-        <v>0.25641025641025644</v>
+        <v>0.5128205128205129</v>
       </c>
       <c r="J40" s="36" t="s">
         <v>382</v>
@@ -16389,16 +16429,20 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M40" s="52" t="s">
-        <v>414</v>
+      <c r="M40" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STL en BRAZO SCARA/DISEÑO FINAL/Cabezal disco/STL/06_separador_electroiman.stl · reemplaza el separador M4 × 25</t>
+        </is>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="37">
         <v>29</v>
       </c>
-      <c r="B41" s="37" t="s">
-        <v>418</v>
+      <c r="B41" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abrazadera M12 del sensor (PLA+)</t>
+        </is>
       </c>
       <c r="C41" s="37" t="s">
         <v>28</v>
@@ -16406,21 +16450,23 @@
       <c r="D41" s="37">
         <v>1</v>
       </c>
-      <c r="E41" s="50"/>
+      <c r="E41" s="50">
+        <v>6.9</v>
+      </c>
       <c r="F41" s="53">
-        <v>4</v>
+        <v>6.1</v>
       </c>
       <c r="G41" s="50">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>6.1</v>
       </c>
       <c r="H41" s="50">
         <f t="shared" si="1"/>
-        <v>0.34188034188034189</v>
+        <v>0.5213675213675214</v>
       </c>
       <c r="I41" s="50">
         <f t="shared" si="2"/>
-        <v>0.34188034188034189</v>
+        <v>0.5213675213675214</v>
       </c>
       <c r="J41" s="36" t="s">
         <v>382</v>
@@ -16430,8 +16476,10 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M41" s="52" t="s">
-        <v>414</v>
+      <c r="M41" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STL en BRAZO SCARA/DISEÑO FINAL/Cabezal disco/STL/07_abrazadera_sensor_M12.stl</t>
+        </is>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>